<commit_message>
added figure ticker labels, and more information for exposure formula
</commit_message>
<xml_diff>
--- a/results/batchruns/batch_kalman_summary.xlsx
+++ b/results/batchruns/batch_kalman_summary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="100" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="320" uniqueCount="54">
   <si>
     <t>Ticker</t>
   </si>
@@ -88,6 +88,93 @@
   </si>
   <si>
     <t>SharpeImprovement</t>
+  </si>
+  <si>
+    <t>BaselineReturnPct</t>
+  </si>
+  <si>
+    <t>ExposureReturnPct</t>
+  </si>
+  <si>
+    <t>BaselineMaxDrawdownPct</t>
+  </si>
+  <si>
+    <t>ExposureMaxDrawdownPct</t>
+  </si>
+  <si>
+    <t>BaselineSharpe</t>
+  </si>
+  <si>
+    <t>ExposureSharpe</t>
+  </si>
+  <si>
+    <t>BuyHoldBuyCount</t>
+  </si>
+  <si>
+    <t>BaselineBuyCount</t>
+  </si>
+  <si>
+    <t>ExposureBuyCount</t>
+  </si>
+  <si>
+    <t>BuyHoldSellCount</t>
+  </si>
+  <si>
+    <t>BaselineSellCount</t>
+  </si>
+  <si>
+    <t>ExposureSellCount</t>
+  </si>
+  <si>
+    <t>BuyHoldTradeCount</t>
+  </si>
+  <si>
+    <t>BaselineTradeCount</t>
+  </si>
+  <si>
+    <t>ExposureTradeCount</t>
+  </si>
+  <si>
+    <t>BuyHoldTimeInMarketPct</t>
+  </si>
+  <si>
+    <t>BaselineTimeInMarketPct</t>
+  </si>
+  <si>
+    <t>ExposureTimeInMarketPct</t>
+  </si>
+  <si>
+    <t>ExposureAveragePct</t>
+  </si>
+  <si>
+    <t>ExposureTurnoverTotal</t>
+  </si>
+  <si>
+    <t>BuyHoldExcessReturnPct</t>
+  </si>
+  <si>
+    <t>BaselineExcessReturnPct</t>
+  </si>
+  <si>
+    <t>ExposureExcessReturnPct</t>
+  </si>
+  <si>
+    <t>BuyHoldDrawdownImprovementPct</t>
+  </si>
+  <si>
+    <t>BaselineDrawdownImprovementPct</t>
+  </si>
+  <si>
+    <t>ExposureDrawdownImprovementPct</t>
+  </si>
+  <si>
+    <t>BuyHoldSharpeImprovement</t>
+  </si>
+  <si>
+    <t>BaselineSharpeImprovement</t>
+  </si>
+  <si>
+    <t>ExposureSharpeImprovement</t>
   </si>
 </sst>
 </file>
@@ -133,7 +220,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:AM6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.83984375" customWidth="true"/>
@@ -143,19 +230,38 @@
     <col min="5" max="5" width="6.9453125" customWidth="true"/>
     <col min="6" max="6" width="14.20703125" customWidth="true"/>
     <col min="7" max="7" width="13.9453125" customWidth="true"/>
-    <col min="8" max="8" width="8.7890625" customWidth="true"/>
-    <col min="9" max="9" width="8.5234375" customWidth="true"/>
-    <col min="10" max="10" width="10.3671875" customWidth="true"/>
-    <col min="11" max="11" width="14.734375" customWidth="true"/>
-    <col min="12" max="12" width="15.41796875" customWidth="true"/>
-    <col min="13" max="13" width="15.5234375" customWidth="true"/>
-    <col min="14" max="14" width="22.20703125" customWidth="true"/>
-    <col min="15" max="15" width="22.3125" customWidth="true"/>
-    <col min="16" max="16" width="13.1015625" customWidth="true"/>
-    <col min="17" max="17" width="13.20703125" customWidth="true"/>
-    <col min="18" max="18" width="13.9453125" customWidth="true"/>
-    <col min="19" max="19" width="22.99609375" customWidth="true"/>
-    <col min="20" max="20" width="17.3671875" customWidth="true"/>
+    <col min="8" max="8" width="15.5234375" customWidth="true"/>
+    <col min="9" max="9" width="15.3671875" customWidth="true"/>
+    <col min="10" max="10" width="16.1015625" customWidth="true"/>
+    <col min="11" max="11" width="22.3125" customWidth="true"/>
+    <col min="12" max="12" width="22.15625" customWidth="true"/>
+    <col min="13" max="13" width="22.89453125" customWidth="true"/>
+    <col min="14" max="14" width="13.20703125" customWidth="true"/>
+    <col min="15" max="15" width="13.05078125" customWidth="true"/>
+    <col min="16" max="16" width="13.7890625" customWidth="true"/>
+    <col min="17" max="17" width="15.41796875" customWidth="true"/>
+    <col min="18" max="18" width="15.26171875" customWidth="true"/>
+    <col min="19" max="19" width="16" customWidth="true"/>
+    <col min="20" max="20" width="15.15625" customWidth="true"/>
+    <col min="21" max="21" width="15" customWidth="true"/>
+    <col min="22" max="22" width="15.734375" customWidth="true"/>
+    <col min="23" max="23" width="16.99609375" customWidth="true"/>
+    <col min="24" max="24" width="16.83984375" customWidth="true"/>
+    <col min="25" max="25" width="17.578125" customWidth="true"/>
+    <col min="26" max="26" width="21.3671875" customWidth="true"/>
+    <col min="27" max="27" width="21.20703125" customWidth="true"/>
+    <col min="28" max="28" width="21.9453125" customWidth="true"/>
+    <col min="29" max="29" width="17.20703125" customWidth="true"/>
+    <col min="30" max="30" width="19.5234375" customWidth="true"/>
+    <col min="31" max="31" width="20.578125" customWidth="true"/>
+    <col min="32" max="32" width="20.41796875" customWidth="true"/>
+    <col min="33" max="33" width="21.15625" customWidth="true"/>
+    <col min="34" max="34" width="29.62890625" customWidth="true"/>
+    <col min="35" max="35" width="29.47265625" customWidth="true"/>
+    <col min="36" max="36" width="30.20703125" customWidth="true"/>
+    <col min="37" max="37" width="23.99609375" customWidth="true"/>
+    <col min="38" max="38" width="23.83984375" customWidth="true"/>
+    <col min="39" max="39" width="24.578125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -181,43 +287,100 @@
         <v>11</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="K1" s="0" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="L1" s="0" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="M1" s="0" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="N1" s="0" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="O1" s="0" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="P1" s="0" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="Q1" s="0" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="R1" s="0" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="S1" s="0" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="T1" s="0" t="s">
-        <v>24</v>
+        <v>34</v>
+      </c>
+      <c r="U1" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="V1" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="X1" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y1" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z1" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA1" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB1" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC1" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="AD1" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="AE1" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="AF1" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="AG1" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="AH1" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI1" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ1" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="AK1" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="AL1" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="AM1" s="0" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="2">
@@ -243,43 +406,100 @@
         <v>8</v>
       </c>
       <c r="H2" s="0">
+        <v>339.63177562489244</v>
+      </c>
+      <c r="I2" s="0">
+        <v>432.28680471328511</v>
+      </c>
+      <c r="J2" s="0">
+        <v>224.50111077957743</v>
+      </c>
+      <c r="K2" s="0">
+        <v>-33.715385820778607</v>
+      </c>
+      <c r="L2" s="0">
+        <v>-24.073604766594158</v>
+      </c>
+      <c r="M2" s="0">
+        <v>-18.049438969990849</v>
+      </c>
+      <c r="N2" s="0">
+        <v>0.82591294677085225</v>
+      </c>
+      <c r="O2" s="0">
+        <v>1.0279386507973149</v>
+      </c>
+      <c r="P2" s="0">
+        <v>0.96967081100248498</v>
+      </c>
+      <c r="Q2" s="0">
+        <v>1</v>
+      </c>
+      <c r="R2" s="0">
         <v>7</v>
       </c>
-      <c r="I2" s="0">
+      <c r="S2" s="0">
+        <v>7</v>
+      </c>
+      <c r="T2" s="0">
+        <v>0</v>
+      </c>
+      <c r="U2" s="0">
         <v>6</v>
       </c>
-      <c r="J2" s="0">
+      <c r="V2" s="0">
+        <v>6</v>
+      </c>
+      <c r="W2" s="0">
+        <v>0</v>
+      </c>
+      <c r="X2" s="0">
         <v>13</v>
       </c>
-      <c r="K2" s="0">
+      <c r="Y2" s="0">
+        <v>381</v>
+      </c>
+      <c r="Z2" s="0">
+        <v>100</v>
+      </c>
+      <c r="AA2" s="0">
         <v>96.652719665271974</v>
       </c>
-      <c r="L2" s="0">
-        <v>432.28680471328511</v>
-      </c>
-      <c r="M2" s="0">
-        <v>339.63177562489244</v>
-      </c>
-      <c r="N2" s="0">
-        <v>-24.073604766594158</v>
-      </c>
-      <c r="O2" s="0">
-        <v>-33.715385820778607</v>
-      </c>
-      <c r="P2" s="0">
-        <v>1.0279386507973149</v>
-      </c>
-      <c r="Q2" s="0">
-        <v>0.82591294677085225</v>
-      </c>
-      <c r="R2" s="0">
-        <v>92.655029088392666</v>
-      </c>
-      <c r="S2" s="0">
-        <v>9.6417810541844489</v>
-      </c>
-      <c r="T2" s="0">
+      <c r="AB2" s="0">
+        <v>96.652719665271974</v>
+      </c>
+      <c r="AC2" s="0">
+        <v>74.677475592747726</v>
+      </c>
+      <c r="AD2" s="0">
+        <v>77.349999999999909</v>
+      </c>
+      <c r="AE2" s="0">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="0">
+        <v>92.655029088392652</v>
+      </c>
+      <c r="AG2" s="0">
+        <v>-115.13066484531502</v>
+      </c>
+      <c r="AH2" s="0">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="0">
+        <v>9.6417810541844506</v>
+      </c>
+      <c r="AJ2" s="0">
+        <v>15.66594685078776</v>
+      </c>
+      <c r="AK2" s="0">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="0">
         <v>0.20202570402646269</v>
+      </c>
+      <c r="AM2" s="0">
+        <v>0.14375786423163273</v>
       </c>
     </row>
     <row r="3">
@@ -305,43 +525,100 @@
         <v>8</v>
       </c>
       <c r="H3" s="0">
+        <v>676.99257536452114</v>
+      </c>
+      <c r="I3" s="0">
+        <v>626.54584561639831</v>
+      </c>
+      <c r="J3" s="0">
+        <v>323.37004908517014</v>
+      </c>
+      <c r="K3" s="0">
+        <v>-35.119666881826539</v>
+      </c>
+      <c r="L3" s="0">
+        <v>-29.257281215398066</v>
+      </c>
+      <c r="M3" s="0">
+        <v>-23.488507889567888</v>
+      </c>
+      <c r="N3" s="0">
+        <v>0.93436024338566648</v>
+      </c>
+      <c r="O3" s="0">
+        <v>1.0074503028125021</v>
+      </c>
+      <c r="P3" s="0">
+        <v>0.96561488668777562</v>
+      </c>
+      <c r="Q3" s="0">
+        <v>1</v>
+      </c>
+      <c r="R3" s="0">
         <v>14</v>
       </c>
-      <c r="I3" s="0">
+      <c r="S3" s="0">
+        <v>14</v>
+      </c>
+      <c r="T3" s="0">
+        <v>0</v>
+      </c>
+      <c r="U3" s="0">
         <v>13</v>
       </c>
-      <c r="J3" s="0">
+      <c r="V3" s="0">
+        <v>13</v>
+      </c>
+      <c r="W3" s="0">
+        <v>0</v>
+      </c>
+      <c r="X3" s="0">
         <v>27</v>
       </c>
-      <c r="K3" s="0">
+      <c r="Y3" s="0">
+        <v>454</v>
+      </c>
+      <c r="Z3" s="0">
+        <v>100</v>
+      </c>
+      <c r="AA3" s="0">
         <v>93.20083682008368</v>
       </c>
-      <c r="L3" s="0">
-        <v>626.54584561639831</v>
-      </c>
-      <c r="M3" s="0">
-        <v>676.99257536452114</v>
-      </c>
-      <c r="N3" s="0">
-        <v>-29.257281215398066</v>
-      </c>
-      <c r="O3" s="0">
-        <v>-35.119666881826539</v>
-      </c>
-      <c r="P3" s="0">
-        <v>1.0074503028125021</v>
-      </c>
-      <c r="Q3" s="0">
-        <v>0.93436024338566648</v>
-      </c>
-      <c r="R3" s="0">
-        <v>-50.446729748122834</v>
-      </c>
-      <c r="S3" s="0">
-        <v>5.862385666428473</v>
-      </c>
-      <c r="T3" s="0">
+      <c r="AB3" s="0">
+        <v>93.20083682008368</v>
+      </c>
+      <c r="AC3" s="0">
+        <v>72.80509065550919</v>
+      </c>
+      <c r="AD3" s="0">
+        <v>95.749999999999829</v>
+      </c>
+      <c r="AE3" s="0">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="0">
+        <v>-50.446729748122806</v>
+      </c>
+      <c r="AG3" s="0">
+        <v>-353.62252627935095</v>
+      </c>
+      <c r="AH3" s="0">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="0">
+        <v>5.8623856664284713</v>
+      </c>
+      <c r="AJ3" s="0">
+        <v>11.63115899225865</v>
+      </c>
+      <c r="AK3" s="0">
+        <v>0</v>
+      </c>
+      <c r="AL3" s="0">
         <v>0.073090059426835663</v>
+      </c>
+      <c r="AM3" s="0">
+        <v>0.031254643302109142</v>
       </c>
     </row>
     <row r="4">
@@ -367,43 +644,100 @@
         <v>8</v>
       </c>
       <c r="H4" s="0">
+        <v>456.72653958944289</v>
+      </c>
+      <c r="I4" s="0">
+        <v>621.94971594098104</v>
+      </c>
+      <c r="J4" s="0">
+        <v>283.64497008926219</v>
+      </c>
+      <c r="K4" s="0">
+        <v>-32.676170186531131</v>
+      </c>
+      <c r="L4" s="0">
+        <v>-24.718937424899057</v>
+      </c>
+      <c r="M4" s="0">
+        <v>-18.91276015811717</v>
+      </c>
+      <c r="N4" s="0">
+        <v>0.85109775601218884</v>
+      </c>
+      <c r="O4" s="0">
+        <v>1.0845880660396914</v>
+      </c>
+      <c r="P4" s="0">
+        <v>0.98200242162032125</v>
+      </c>
+      <c r="Q4" s="0">
+        <v>1</v>
+      </c>
+      <c r="R4" s="0">
         <v>9</v>
       </c>
-      <c r="I4" s="0">
+      <c r="S4" s="0">
+        <v>9</v>
+      </c>
+      <c r="T4" s="0">
+        <v>0</v>
+      </c>
+      <c r="U4" s="0">
         <v>8</v>
       </c>
-      <c r="J4" s="0">
+      <c r="V4" s="0">
+        <v>8</v>
+      </c>
+      <c r="W4" s="0">
+        <v>0</v>
+      </c>
+      <c r="X4" s="0">
         <v>17</v>
       </c>
-      <c r="K4" s="0">
+      <c r="Y4" s="0">
+        <v>420</v>
+      </c>
+      <c r="Z4" s="0">
+        <v>100</v>
+      </c>
+      <c r="AA4" s="0">
         <v>94.735006973500703</v>
       </c>
-      <c r="L4" s="0">
-        <v>621.94971594098104</v>
-      </c>
-      <c r="M4" s="0">
-        <v>456.72653958944289</v>
-      </c>
-      <c r="N4" s="0">
-        <v>-24.718937424899057</v>
-      </c>
-      <c r="O4" s="0">
-        <v>-32.676170186531131</v>
-      </c>
-      <c r="P4" s="0">
-        <v>1.0845880660396914</v>
-      </c>
-      <c r="Q4" s="0">
-        <v>0.85109775601218884</v>
-      </c>
-      <c r="R4" s="0">
-        <v>165.22317635153814</v>
-      </c>
-      <c r="S4" s="0">
-        <v>7.9572327616320742</v>
-      </c>
-      <c r="T4" s="0">
+      <c r="AB4" s="0">
+        <v>94.735006973500703</v>
+      </c>
+      <c r="AC4" s="0">
+        <v>73.540794979079649</v>
+      </c>
+      <c r="AD4" s="0">
+        <v>85.849999999999881</v>
+      </c>
+      <c r="AE4" s="0">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="0">
+        <v>165.22317635153811</v>
+      </c>
+      <c r="AG4" s="0">
+        <v>-173.08156950018073</v>
+      </c>
+      <c r="AH4" s="0">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="0">
+        <v>7.9572327616320715</v>
+      </c>
+      <c r="AJ4" s="0">
+        <v>13.763410028413958</v>
+      </c>
+      <c r="AK4" s="0">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="0">
         <v>0.23349031002750253</v>
+      </c>
+      <c r="AM4" s="0">
+        <v>0.13090466560813241</v>
       </c>
     </row>
     <row r="5">
@@ -429,43 +763,100 @@
         <v>8</v>
       </c>
       <c r="H5" s="0">
+        <v>1019.949394325786</v>
+      </c>
+      <c r="I5" s="0">
+        <v>688.78812976136112</v>
+      </c>
+      <c r="J5" s="0">
+        <v>294.96246074901319</v>
+      </c>
+      <c r="K5" s="0">
+        <v>-37.148247930078625</v>
+      </c>
+      <c r="L5" s="0">
+        <v>-40.423911859135252</v>
+      </c>
+      <c r="M5" s="0">
+        <v>-35.187983579073709</v>
+      </c>
+      <c r="N5" s="0">
+        <v>0.91899963490511405</v>
+      </c>
+      <c r="O5" s="0">
+        <v>0.87755309505140477</v>
+      </c>
+      <c r="P5" s="0">
+        <v>0.74169326182186202</v>
+      </c>
+      <c r="Q5" s="0">
+        <v>1</v>
+      </c>
+      <c r="R5" s="0">
         <v>21</v>
       </c>
-      <c r="I5" s="0">
+      <c r="S5" s="0">
+        <v>21</v>
+      </c>
+      <c r="T5" s="0">
+        <v>0</v>
+      </c>
+      <c r="U5" s="0">
         <v>20</v>
       </c>
-      <c r="J5" s="0">
+      <c r="V5" s="0">
+        <v>20</v>
+      </c>
+      <c r="W5" s="0">
+        <v>0</v>
+      </c>
+      <c r="X5" s="0">
         <v>41</v>
       </c>
-      <c r="K5" s="0">
+      <c r="Y5" s="0">
+        <v>534</v>
+      </c>
+      <c r="Z5" s="0">
+        <v>100</v>
+      </c>
+      <c r="AA5" s="0">
         <v>90.202231520223151</v>
       </c>
-      <c r="L5" s="0">
-        <v>688.78812976136112</v>
-      </c>
-      <c r="M5" s="0">
-        <v>1019.949394325786</v>
-      </c>
-      <c r="N5" s="0">
-        <v>-40.423911859135252</v>
-      </c>
-      <c r="O5" s="0">
-        <v>-37.148247930078625</v>
-      </c>
-      <c r="P5" s="0">
-        <v>0.87755309505140477</v>
-      </c>
-      <c r="Q5" s="0">
-        <v>0.91899963490511405</v>
-      </c>
-      <c r="R5" s="0">
+      <c r="AB5" s="0">
+        <v>90.202231520223151</v>
+      </c>
+      <c r="AC5" s="0">
+        <v>70.313807531380817</v>
+      </c>
+      <c r="AD5" s="0">
+        <v>116.19999999999978</v>
+      </c>
+      <c r="AE5" s="0">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="0">
         <v>-331.16126456442487</v>
       </c>
-      <c r="S5" s="0">
+      <c r="AG5" s="0">
+        <v>-724.9869335767728</v>
+      </c>
+      <c r="AH5" s="0">
+        <v>0</v>
+      </c>
+      <c r="AI5" s="0">
         <v>-3.275663929056627</v>
       </c>
-      <c r="T5" s="0">
+      <c r="AJ5" s="0">
+        <v>1.9602643510049145</v>
+      </c>
+      <c r="AK5" s="0">
+        <v>0</v>
+      </c>
+      <c r="AL5" s="0">
         <v>-0.041446539853709274</v>
+      </c>
+      <c r="AM5" s="0">
+        <v>-0.17730637308325203</v>
       </c>
     </row>
     <row r="6">
@@ -491,43 +882,100 @@
         <v>8</v>
       </c>
       <c r="H6" s="0">
+        <v>43601.969744949427</v>
+      </c>
+      <c r="I6" s="0">
+        <v>9324.8638502783724</v>
+      </c>
+      <c r="J6" s="0">
+        <v>3897.5280797971905</v>
+      </c>
+      <c r="K6" s="0">
+        <v>-66.335097234686927</v>
+      </c>
+      <c r="L6" s="0">
+        <v>-57.006738721462568</v>
+      </c>
+      <c r="M6" s="0">
+        <v>-51.719621905494904</v>
+      </c>
+      <c r="N6" s="0">
+        <v>1.3464882956134154</v>
+      </c>
+      <c r="O6" s="0">
+        <v>1.1506600623020915</v>
+      </c>
+      <c r="P6" s="0">
+        <v>1.1293807135969574</v>
+      </c>
+      <c r="Q6" s="0">
+        <v>1</v>
+      </c>
+      <c r="R6" s="0">
         <v>41</v>
       </c>
-      <c r="I6" s="0">
+      <c r="S6" s="0">
+        <v>41</v>
+      </c>
+      <c r="T6" s="0">
+        <v>0</v>
+      </c>
+      <c r="U6" s="0">
         <v>40</v>
       </c>
-      <c r="J6" s="0">
+      <c r="V6" s="0">
+        <v>40</v>
+      </c>
+      <c r="W6" s="0">
+        <v>0</v>
+      </c>
+      <c r="X6" s="0">
         <v>81</v>
       </c>
-      <c r="K6" s="0">
+      <c r="Y6" s="0">
+        <v>601</v>
+      </c>
+      <c r="Z6" s="0">
+        <v>100</v>
+      </c>
+      <c r="AA6" s="0">
         <v>84.10041841004184</v>
       </c>
-      <c r="L6" s="0">
-        <v>9324.8638502783724</v>
-      </c>
-      <c r="M6" s="0">
-        <v>43601.969744949427</v>
-      </c>
-      <c r="N6" s="0">
-        <v>-57.006738721462568</v>
-      </c>
-      <c r="O6" s="0">
-        <v>-66.335097234686927</v>
-      </c>
-      <c r="P6" s="0">
-        <v>1.1506600623020915</v>
-      </c>
-      <c r="Q6" s="0">
-        <v>1.3464882956134154</v>
-      </c>
-      <c r="R6" s="0">
+      <c r="AB6" s="0">
+        <v>84.10041841004184</v>
+      </c>
+      <c r="AC6" s="0">
+        <v>67.313458856345903</v>
+      </c>
+      <c r="AD6" s="0">
+        <v>152.59999999999982</v>
+      </c>
+      <c r="AE6" s="0">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="0">
         <v>-34277.105894671055</v>
       </c>
-      <c r="S6" s="0">
-        <v>9.3283585132243587</v>
-      </c>
-      <c r="T6" s="0">
+      <c r="AG6" s="0">
+        <v>-39704.441665152241</v>
+      </c>
+      <c r="AH6" s="0">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="0">
+        <v>9.3283585132243552</v>
+      </c>
+      <c r="AJ6" s="0">
+        <v>14.615475329192018</v>
+      </c>
+      <c r="AK6" s="0">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="0">
         <v>-0.19582823331132393</v>
+      </c>
+      <c r="AM6" s="0">
+        <v>-0.21710758201645808</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V4: at or below baseline
</commit_message>
<xml_diff>
--- a/results/batchruns/batch_kalman_summary.xlsx
+++ b/results/batchruns/batch_kalman_summary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="320" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="408" uniqueCount="54">
   <si>
     <t>Ticker</t>
   </si>
@@ -412,7 +412,7 @@
         <v>432.28680471328511</v>
       </c>
       <c r="J2" s="0">
-        <v>224.50111077957743</v>
+        <v>389.35213716591255</v>
       </c>
       <c r="K2" s="0">
         <v>-33.715385820778607</v>
@@ -421,7 +421,7 @@
         <v>-24.073604766594158</v>
       </c>
       <c r="M2" s="0">
-        <v>-18.049438969990849</v>
+        <v>-24.894281809042027</v>
       </c>
       <c r="N2" s="0">
         <v>0.82591294677085225</v>
@@ -430,7 +430,7 @@
         <v>1.0279386507973149</v>
       </c>
       <c r="P2" s="0">
-        <v>0.96967081100248498</v>
+        <v>0.99587018398945515</v>
       </c>
       <c r="Q2" s="0">
         <v>1</v>
@@ -457,7 +457,7 @@
         <v>13</v>
       </c>
       <c r="Y2" s="0">
-        <v>381</v>
+        <v>45</v>
       </c>
       <c r="Z2" s="0">
         <v>100</v>
@@ -469,10 +469,10 @@
         <v>96.652719665271974</v>
       </c>
       <c r="AC2" s="0">
-        <v>74.677475592747726</v>
+        <v>96.103556485355639</v>
       </c>
       <c r="AD2" s="0">
-        <v>77.349999999999909</v>
+        <v>19</v>
       </c>
       <c r="AE2" s="0">
         <v>0</v>
@@ -481,7 +481,7 @@
         <v>92.655029088392652</v>
       </c>
       <c r="AG2" s="0">
-        <v>-115.13066484531502</v>
+        <v>49.720361541020083</v>
       </c>
       <c r="AH2" s="0">
         <v>0</v>
@@ -490,7 +490,7 @@
         <v>9.6417810541844506</v>
       </c>
       <c r="AJ2" s="0">
-        <v>15.66594685078776</v>
+        <v>8.8211040117365798</v>
       </c>
       <c r="AK2" s="0">
         <v>0</v>
@@ -499,7 +499,7 @@
         <v>0.20202570402646269</v>
       </c>
       <c r="AM2" s="0">
-        <v>0.14375786423163273</v>
+        <v>0.1699572372186029</v>
       </c>
     </row>
     <row r="3">
@@ -531,7 +531,7 @@
         <v>626.54584561639831</v>
       </c>
       <c r="J3" s="0">
-        <v>323.37004908517014</v>
+        <v>590.27138604251502</v>
       </c>
       <c r="K3" s="0">
         <v>-35.119666881826539</v>
@@ -540,7 +540,7 @@
         <v>-29.257281215398066</v>
       </c>
       <c r="M3" s="0">
-        <v>-23.488507889567888</v>
+        <v>-27.8097265711462</v>
       </c>
       <c r="N3" s="0">
         <v>0.93436024338566648</v>
@@ -549,7 +549,7 @@
         <v>1.0074503028125021</v>
       </c>
       <c r="P3" s="0">
-        <v>0.96561488668777562</v>
+        <v>1.0059736916901678</v>
       </c>
       <c r="Q3" s="0">
         <v>1</v>
@@ -576,7 +576,7 @@
         <v>27</v>
       </c>
       <c r="Y3" s="0">
-        <v>454</v>
+        <v>92</v>
       </c>
       <c r="Z3" s="0">
         <v>100</v>
@@ -588,10 +588,10 @@
         <v>93.20083682008368</v>
       </c>
       <c r="AC3" s="0">
-        <v>72.80509065550919</v>
+        <v>92.154811715481173</v>
       </c>
       <c r="AD3" s="0">
-        <v>95.749999999999829</v>
+        <v>38</v>
       </c>
       <c r="AE3" s="0">
         <v>0</v>
@@ -600,7 +600,7 @@
         <v>-50.446729748122806</v>
       </c>
       <c r="AG3" s="0">
-        <v>-353.62252627935095</v>
+        <v>-86.721189322006069</v>
       </c>
       <c r="AH3" s="0">
         <v>0</v>
@@ -609,7 +609,7 @@
         <v>5.8623856664284713</v>
       </c>
       <c r="AJ3" s="0">
-        <v>11.63115899225865</v>
+        <v>7.3099403106803411</v>
       </c>
       <c r="AK3" s="0">
         <v>0</v>
@@ -618,7 +618,7 @@
         <v>0.073090059426835663</v>
       </c>
       <c r="AM3" s="0">
-        <v>0.031254643302109142</v>
+        <v>0.071613448304501337</v>
       </c>
     </row>
     <row r="4">
@@ -650,7 +650,7 @@
         <v>621.94971594098104</v>
       </c>
       <c r="J4" s="0">
-        <v>283.64497008926219</v>
+        <v>578.79773301908415</v>
       </c>
       <c r="K4" s="0">
         <v>-32.676170186531131</v>
@@ -659,7 +659,7 @@
         <v>-24.718937424899057</v>
       </c>
       <c r="M4" s="0">
-        <v>-18.91276015811717</v>
+        <v>-23.015392999535035</v>
       </c>
       <c r="N4" s="0">
         <v>0.85109775601218884</v>
@@ -668,7 +668,7 @@
         <v>1.0845880660396914</v>
       </c>
       <c r="P4" s="0">
-        <v>0.98200242162032125</v>
+        <v>1.074585887859431</v>
       </c>
       <c r="Q4" s="0">
         <v>1</v>
@@ -695,7 +695,7 @@
         <v>17</v>
       </c>
       <c r="Y4" s="0">
-        <v>420</v>
+        <v>70</v>
       </c>
       <c r="Z4" s="0">
         <v>100</v>
@@ -707,10 +707,10 @@
         <v>94.735006973500703</v>
       </c>
       <c r="AC4" s="0">
-        <v>73.540794979079649</v>
+        <v>93.976638772663875</v>
       </c>
       <c r="AD4" s="0">
-        <v>85.849999999999881</v>
+        <v>27</v>
       </c>
       <c r="AE4" s="0">
         <v>0</v>
@@ -719,7 +719,7 @@
         <v>165.22317635153811</v>
       </c>
       <c r="AG4" s="0">
-        <v>-173.08156950018073</v>
+        <v>122.07119342964123</v>
       </c>
       <c r="AH4" s="0">
         <v>0</v>
@@ -728,7 +728,7 @@
         <v>7.9572327616320715</v>
       </c>
       <c r="AJ4" s="0">
-        <v>13.763410028413958</v>
+        <v>9.6607771869960946</v>
       </c>
       <c r="AK4" s="0">
         <v>0</v>
@@ -737,7 +737,7 @@
         <v>0.23349031002750253</v>
       </c>
       <c r="AM4" s="0">
-        <v>0.13090466560813241</v>
+        <v>0.22348813184724214</v>
       </c>
     </row>
     <row r="5">
@@ -769,7 +769,7 @@
         <v>688.78812976136112</v>
       </c>
       <c r="J5" s="0">
-        <v>294.96246074901319</v>
+        <v>675.19580525579477</v>
       </c>
       <c r="K5" s="0">
         <v>-37.148247930078625</v>
@@ -778,7 +778,7 @@
         <v>-40.423911859135252</v>
       </c>
       <c r="M5" s="0">
-        <v>-35.187983579073709</v>
+        <v>-40.108032302072431</v>
       </c>
       <c r="N5" s="0">
         <v>0.91899963490511405</v>
@@ -787,7 +787,7 @@
         <v>0.87755309505140477</v>
       </c>
       <c r="P5" s="0">
-        <v>0.74169326182186202</v>
+        <v>0.88498222039579366</v>
       </c>
       <c r="Q5" s="0">
         <v>1</v>
@@ -814,7 +814,7 @@
         <v>41</v>
       </c>
       <c r="Y5" s="0">
-        <v>534</v>
+        <v>127</v>
       </c>
       <c r="Z5" s="0">
         <v>100</v>
@@ -826,10 +826,10 @@
         <v>90.202231520223151</v>
       </c>
       <c r="AC5" s="0">
-        <v>70.313807531380817</v>
+        <v>88.70292887029288</v>
       </c>
       <c r="AD5" s="0">
-        <v>116.19999999999978</v>
+        <v>54</v>
       </c>
       <c r="AE5" s="0">
         <v>0</v>
@@ -838,7 +838,7 @@
         <v>-331.16126456442487</v>
       </c>
       <c r="AG5" s="0">
-        <v>-724.9869335767728</v>
+        <v>-344.75358906999122</v>
       </c>
       <c r="AH5" s="0">
         <v>0</v>
@@ -847,7 +847,7 @@
         <v>-3.275663929056627</v>
       </c>
       <c r="AJ5" s="0">
-        <v>1.9602643510049145</v>
+        <v>-2.9597843719938011</v>
       </c>
       <c r="AK5" s="0">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>-0.041446539853709274</v>
       </c>
       <c r="AM5" s="0">
-        <v>-0.17730637308325203</v>
+        <v>-0.034017414509320387</v>
       </c>
     </row>
     <row r="6">
@@ -888,7 +888,7 @@
         <v>9324.8638502783724</v>
       </c>
       <c r="J6" s="0">
-        <v>3897.5280797971905</v>
+        <v>9488.7380277611574</v>
       </c>
       <c r="K6" s="0">
         <v>-66.335097234686927</v>
@@ -897,7 +897,7 @@
         <v>-57.006738721462568</v>
       </c>
       <c r="M6" s="0">
-        <v>-51.719621905494904</v>
+        <v>-55.131649243972333</v>
       </c>
       <c r="N6" s="0">
         <v>1.3464882956134154</v>
@@ -906,7 +906,7 @@
         <v>1.1506600623020915</v>
       </c>
       <c r="P6" s="0">
-        <v>1.1293807135969574</v>
+        <v>1.1818983053288856</v>
       </c>
       <c r="Q6" s="0">
         <v>1</v>
@@ -933,7 +933,7 @@
         <v>81</v>
       </c>
       <c r="Y6" s="0">
-        <v>601</v>
+        <v>217</v>
       </c>
       <c r="Z6" s="0">
         <v>100</v>
@@ -945,10 +945,10 @@
         <v>84.10041841004184</v>
       </c>
       <c r="AC6" s="0">
-        <v>67.313458856345903</v>
+        <v>81.459205020920507</v>
       </c>
       <c r="AD6" s="0">
-        <v>152.59999999999982</v>
+        <v>97.5</v>
       </c>
       <c r="AE6" s="0">
         <v>0</v>
@@ -957,7 +957,7 @@
         <v>-34277.105894671055</v>
       </c>
       <c r="AG6" s="0">
-        <v>-39704.441665152241</v>
+        <v>-34113.231717188275</v>
       </c>
       <c r="AH6" s="0">
         <v>0</v>
@@ -966,7 +966,7 @@
         <v>9.3283585132243552</v>
       </c>
       <c r="AJ6" s="0">
-        <v>14.615475329192018</v>
+        <v>11.203447990714588</v>
       </c>
       <c r="AK6" s="0">
         <v>0</v>
@@ -975,7 +975,7 @@
         <v>-0.19582823331132393</v>
       </c>
       <c r="AM6" s="0">
-        <v>-0.21710758201645808</v>
+        <v>-0.16458999028452981</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated file naming scheme for wf files; also, ran new tests on exposure formula by changing r_meas: results are improving slightly.
</commit_message>
<xml_diff>
--- a/results/batchruns/batch_kalman_summary.xlsx
+++ b/results/batchruns/batch_kalman_summary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="408" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="534" uniqueCount="54">
   <si>
     <t>Ticker</t>
   </si>
@@ -412,7 +412,7 @@
         <v>432.28680471328511</v>
       </c>
       <c r="J2" s="0">
-        <v>389.35213716591255</v>
+        <v>390.80222452081006</v>
       </c>
       <c r="K2" s="0">
         <v>-33.715385820778607</v>
@@ -421,7 +421,7 @@
         <v>-24.073604766594158</v>
       </c>
       <c r="M2" s="0">
-        <v>-24.894281809042027</v>
+        <v>-24.595634948767973</v>
       </c>
       <c r="N2" s="0">
         <v>0.82591294677085225</v>
@@ -430,7 +430,7 @@
         <v>1.0279386507973149</v>
       </c>
       <c r="P2" s="0">
-        <v>0.99587018398945515</v>
+        <v>1.0003024077799496</v>
       </c>
       <c r="Q2" s="0">
         <v>1</v>
@@ -469,7 +469,7 @@
         <v>96.652719665271974</v>
       </c>
       <c r="AC2" s="0">
-        <v>96.103556485355639</v>
+        <v>95.894351464435147</v>
       </c>
       <c r="AD2" s="0">
         <v>19</v>
@@ -481,7 +481,7 @@
         <v>92.655029088392652</v>
       </c>
       <c r="AG2" s="0">
-        <v>49.720361541020083</v>
+        <v>51.170448895917616</v>
       </c>
       <c r="AH2" s="0">
         <v>0</v>
@@ -490,7 +490,7 @@
         <v>9.6417810541844506</v>
       </c>
       <c r="AJ2" s="0">
-        <v>8.8211040117365798</v>
+        <v>9.1197508720106342</v>
       </c>
       <c r="AK2" s="0">
         <v>0</v>
@@ -499,7 +499,7 @@
         <v>0.20202570402646269</v>
       </c>
       <c r="AM2" s="0">
-        <v>0.1699572372186029</v>
+        <v>0.17438946100909736</v>
       </c>
     </row>
     <row r="3">
@@ -531,7 +531,7 @@
         <v>626.54584561639831</v>
       </c>
       <c r="J3" s="0">
-        <v>590.27138604251502</v>
+        <v>562.3751544810583</v>
       </c>
       <c r="K3" s="0">
         <v>-35.119666881826539</v>
@@ -540,7 +540,7 @@
         <v>-29.257281215398066</v>
       </c>
       <c r="M3" s="0">
-        <v>-27.8097265711462</v>
+        <v>-27.996996738255795</v>
       </c>
       <c r="N3" s="0">
         <v>0.93436024338566648</v>
@@ -549,7 +549,7 @@
         <v>1.0074503028125021</v>
       </c>
       <c r="P3" s="0">
-        <v>1.0059736916901678</v>
+        <v>0.99033474459155635</v>
       </c>
       <c r="Q3" s="0">
         <v>1</v>
@@ -588,7 +588,7 @@
         <v>93.20083682008368</v>
       </c>
       <c r="AC3" s="0">
-        <v>92.154811715481173</v>
+        <v>91.771269177126911</v>
       </c>
       <c r="AD3" s="0">
         <v>38</v>
@@ -600,7 +600,7 @@
         <v>-50.446729748122806</v>
       </c>
       <c r="AG3" s="0">
-        <v>-86.721189322006069</v>
+        <v>-114.61742088346281</v>
       </c>
       <c r="AH3" s="0">
         <v>0</v>
@@ -609,7 +609,7 @@
         <v>5.8623856664284713</v>
       </c>
       <c r="AJ3" s="0">
-        <v>7.3099403106803411</v>
+        <v>7.1226701435707422</v>
       </c>
       <c r="AK3" s="0">
         <v>0</v>
@@ -618,7 +618,7 @@
         <v>0.073090059426835663</v>
       </c>
       <c r="AM3" s="0">
-        <v>0.071613448304501337</v>
+        <v>0.055974501205889871</v>
       </c>
     </row>
     <row r="4">
@@ -650,7 +650,7 @@
         <v>621.94971594098104</v>
       </c>
       <c r="J4" s="0">
-        <v>578.79773301908415</v>
+        <v>566.14243367339611</v>
       </c>
       <c r="K4" s="0">
         <v>-32.676170186531131</v>
@@ -659,7 +659,7 @@
         <v>-24.718937424899057</v>
       </c>
       <c r="M4" s="0">
-        <v>-23.015392999535035</v>
+        <v>-23.044707249595898</v>
       </c>
       <c r="N4" s="0">
         <v>0.85109775601218884</v>
@@ -668,7 +668,7 @@
         <v>1.0845880660396914</v>
       </c>
       <c r="P4" s="0">
-        <v>1.074585887859431</v>
+        <v>1.0693447543194616</v>
       </c>
       <c r="Q4" s="0">
         <v>1</v>
@@ -707,7 +707,7 @@
         <v>94.735006973500703</v>
       </c>
       <c r="AC4" s="0">
-        <v>93.976638772663875</v>
+        <v>93.627963737796378</v>
       </c>
       <c r="AD4" s="0">
         <v>27</v>
@@ -719,7 +719,7 @@
         <v>165.22317635153811</v>
       </c>
       <c r="AG4" s="0">
-        <v>122.07119342964123</v>
+        <v>109.41589408395318</v>
       </c>
       <c r="AH4" s="0">
         <v>0</v>
@@ -728,7 +728,7 @@
         <v>7.9572327616320715</v>
       </c>
       <c r="AJ4" s="0">
-        <v>9.6607771869960946</v>
+        <v>9.6314629369352307</v>
       </c>
       <c r="AK4" s="0">
         <v>0</v>
@@ -737,7 +737,7 @@
         <v>0.23349031002750253</v>
       </c>
       <c r="AM4" s="0">
-        <v>0.22348813184724214</v>
+        <v>0.21824699830727279</v>
       </c>
     </row>
     <row r="5">

</xml_diff>